<commit_message>
Apply business answers to TTZV-6011 test checklist
Bonds valued at nominal; mid-period averaging, FX conversion, account-type
scope and BRD documentation gaps excluded; Jira numbers confirmed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149r7b5293oK3v6EmbinnuA
</commit_message>
<xml_diff>
--- a/TTZV-6011_Test_Checklist.xlsx
+++ b/TTZV-6011_Test_Checklist.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Բաց հարցեր" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Թեստային դեպքեր'!$A$1:$O$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Թեստային դեպքեր'!$A$1:$O$29</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="275">
   <si>
     <t xml:space="preserve">Թեստավորման ստուգաթերթ – PLUS CLUB, PLUS DIGITAL, STATUS փաթեթների միջին մնացորդի հաշվարկի մեջ պարտատոմսի հաշվի մնացորդի ներառում</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Հայտ (BRD)</t>
   </si>
   <si>
-    <t xml:space="preserve">TTZV-6011 (PDF-ում՝ «TTZV-60111», տողատակի համարը կցված է)</t>
+    <t xml:space="preserve">TTZV-6011</t>
   </si>
   <si>
     <t xml:space="preserve">Հիմնական լուծում (կապված BRD)</t>
@@ -66,6 +66,12 @@
     <t xml:space="preserve">Պարտատոմսի հաշվի ներառում միջին մնացորդի հաշվարկում</t>
   </si>
   <si>
+    <t xml:space="preserve">Պարտատոմսի հաշվառման արժեք</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Անվանական արժեք (համաձայնեցված 16.10.2026, տես «Բաց հարցեր» Q2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Թեստային միջավայր</t>
   </si>
   <si>
@@ -168,7 +174,7 @@
     <t xml:space="preserve">Թեստային տվյալներ</t>
   </si>
   <si>
-    <t xml:space="preserve">Բոլոր գումարները ՀՀԴ են։ «Միջին մնացորդ»-ը վերջին 3 ամսվա միջինն է։ Պարզության համար թեստային տվյալներում մնացորդները պահել հաստատուն ամբողջ ժամանակահատվածում, եթե դեպքը այլ բան չի պահանջում։</t>
+    <t xml:space="preserve">Բոլոր գումարները ՀՀԴ են։ «Միջին մնացորդ»-ը վերջին 3 ամսվա միջինն է։ Պարտատոմսի գումարները նշված են անվանական արժեքով։ Պարզության համար թեստային տվյալներում մնացորդները պահել հաստատուն ամբողջ ժամանակահատվածում, եթե դեպքը այլ բան չի պահանջում։</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -234,7 +240,7 @@
     <t xml:space="preserve">Գործարկել ամսական հաշվարկը (1-ին աշխատանքային օրվա ռեժիմով) թեստային հաճախորդի համար։ Բացել հաշվարկի արդյունքը / log-ը և գանձման գործարքը LSoft-ում։ Համեմատել հաշվարկված միջին մնացորդը ձեռքով հաշվարկի հետ։</t>
   </si>
   <si>
-    <t xml:space="preserve">Միջին մնացորդ = ցպահանջ + ժամկետային + պարտատոմսի հաշիվների միջին մնացորդների գումարը։ Պարտատոմսի հաշիվը երևում է հաշվարկում ներառված հաշիվների ցանկում։</t>
+    <t xml:space="preserve">Միջին մնացորդ = ցպահանջ + ժամկետային + պարտատոմսի հաշիվների միջին մնացորդների գումարը (պարտատոմսը՝ անվանական արժեքով)։ Պարտատոմսի հաշիվը երևում է հաշվարկում ներառված հաշիվների ցանկում։</t>
   </si>
   <si>
     <t xml:space="preserve">Պարտատոմսի հաշիվը ներառված է հաշվարկում (հիմնական ընդունման չափանիշ)</t>
@@ -441,288 +447,246 @@
     <t xml:space="preserve">C. Պարտատոմսի առանձնահատկություններ</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §1 (միջին մնացորդ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պարտատոմսի հաշիվը բացվել է 3 ամսյա ժամանակահատվածի միջնամասում (օր. վերջին ամսում)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պարտատոմսի մնացորդը միջինում հաշվառվում է միայն փաստացի պահման օրերի համար՝ նույն մեթոդաբանությամբ, ինչ ավանդային հաշիվներինը (տես Բաց հարց Q1)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Միջինացման ճշգրտություն</t>
+    <t xml:space="preserve">Որոշում 16.10.2026 (Q2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLUS CLUB հաճախորդ․ ավանդներ՝ 1,000,000 + պարտատոմս՝ անվանական արժեք 1,000,000, ձեռքբերման / շուկայական արժեք 980,000։ Աշխատավարձ չկա։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Պարտատոմսը հաշվառվում է անվանական արժեքով՝ 1,000,000 → միջին մնացորդ = 2,000,000 ≥ 2,000,000 → Քայլ 2 → վճար 5,000 ՀՀԴ (ձեռքբերման արժեքով կլիներ 1,980,000 → Քայլ 3)։ Կուտակված արժեկտրոնը չի ավելացվում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Պարտատոմսը հաշվառվում է անվանական արժեքով</t>
   </si>
   <si>
     <t xml:space="preserve">TC-15</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պարտատոմսը մարվել / հաշիվը փակվել է ժամանակահատվածի ընթացքում։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Մնացորդը հաշվառվում է մինչև մարման / փակման ամսաթիվը, դրանից հետո՝ 0։ Հաշվարկը չի ընդհատվում սխալով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Մարված պարտատոմսի ճիշտ մշակում</t>
+    <t xml:space="preserve">Միջին</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRD TTZV-6011 §2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդն ունի 2 և ավելի պարտատոմսի հաշիվ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բոլոր պարտատոմսի հաշիվների մնացորդները գումարվում են։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բազմակի պարտատոմսեր</t>
   </si>
   <si>
     <t xml:space="preserve">TC-16</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պարտատոմս արտարժույթով (USD և/կամ EUR)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Մնացորդը փոխարկվում է ՀՀԴ-ի նույն փոխարժեքով և նույն ամսաթվով, ինչ արտարժութային ավանդները (տես Բաց հարց Q3)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Արտարժութային պարտատոմսեր</t>
+    <t xml:space="preserve">Պարտատոմսի հաշիվ՝ 0 մնացորդով կամ փակված մինչև ժամանակահատվածը։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Արդյունքը նույնն է, ինչ առանց պարտատոմսի հաշվի։ Սխալ չկա։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Դատարկ / փակ հաշիվներ</t>
   </si>
   <si>
     <t xml:space="preserve">TC-17</t>
   </si>
   <si>
-    <t xml:space="preserve">Միջին</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդն ունի 2 և ավելի պարտատոմսի հաշիվ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բոլոր պարտատոմսի հաշիվների մնացորդները գումարվում են։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բազմակի պարտատոմսեր</t>
+    <t xml:space="preserve">BRD TTZV-6011 §9 («հաճախորդի՝ պարտատոմսի հաշիվը»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Պարտատոմսի հաշիվ, որը պատկանում է այլ հաճախորդի (օր. փոխկապակցված անձ, երրորդ անձ)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Այլ հաճախորդի պարտատոմսը ՉԻ ներառվում թեստային հաճախորդի հաշվարկում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Միայն հաճախորդի սեփական հաշիվները</t>
   </si>
   <si>
     <t xml:space="preserve">TC-18</t>
   </si>
   <si>
-    <t xml:space="preserve">Պարտատոմսի հաշիվ՝ 0 մնացորդով կամ փակված մինչև ժամանակահատվածը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Արդյունքը նույնն է, ինչ առանց պարտատոմսի հաշվի։ Սխալ չկա։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Դատարկ / փակ հաշիվներ</t>
+    <t xml:space="preserve">D. Գանձում և ելքային տվյալներ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 Քայլ 1–3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-03–TC-08 դեպքերի հաճախորդները։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ստուգել LSoft-ում գանձման գործարքները։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գանձված գումարը համապատասխանում է ակնկալվողին, ճիշտ հաշվից, ճիշտ ամսաթվով (ամսվա 1-ին աշխատանքային օր), ճիշտ գործարքի նկարագրությամբ։ Կրկնակի գանձում չկա։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Վերջնական ֆինանսական արդյունքի ճշգրտություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-19</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §9 («հաճախորդի՝ պարտատոմսի հաշիվը»)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պարտատոմսի հաշիվ, որը պատկանում է այլ հաճախորդի (օր. փոխկապակցված անձ, երրորդ անձ)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Այլ հաճախորդի պարտատոմսը ՉԻ ներառվում թեստային հաճախորդի հաշվարկում։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Միայն հաճախորդի սեփական հաշիվները</t>
+    <t xml:space="preserve">TTZV-4447 STATUS Քայլ 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդների խումբ՝ պարտատոմսով որակավորվող և չորակավորվող։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ստուգել ՍԾՎ/ՍԾԶՎ-ին տրամադրվող անհամապատասխան հաճախորդների ցուցակը։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ցուցակում ներառված են միայն այն հաճախորդները, որոնք պարտատոմսը հաշվի առնելով էլ չեն համապատասխանում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Արտահանման ճշգրտություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-20</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §1 (Scope)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ստուգել, որ ներառվում են ՄԻԱՅՆ պարտատոմսի հաշիվների համար համաձայնեցված հաշվի տեսակները / հաշվեկշռային հաշիվները (տես Q4), և չեն ներառվում այլ ոչ ավանդային հաշիվներ (վարկային, քարտային վարկային գիծ և այլն)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաշվարկում ներառված են միայն ցպահանջ, ժամկետային և պարտատոմսի հաշիվները։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Շրջանակի ճշգրտություն</t>
+    <t xml:space="preserve">TTZV-4447 Scope (ծանուցում)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդներ, որոնք որակավորվում են միայն պարտատոմսի շնորհիվ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ստուգել ծանուցումների ուղարկման log-ը և ՍԾԶՎ-ին տրամադրվող ցուցակը։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Այդ հաճախորդները ծանուցում ՉԵՆ ստանում և ցուցակում ներառված չեն։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդի հաղորդակցության ճշգրտություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-21</t>
   </si>
   <si>
-    <t xml:space="preserve">D. Գանձում և ելքային տվյալներ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 Քայլ 1–3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-03–TC-08 դեպքերի հաճախորդները։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ստուգել LSoft-ում գանձման գործարքները։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գանձված գումարը համապատասխանում է ակնկալվողին, ճիշտ հաշվից, ճիշտ ամսաթվով (ամսվա 1-ին աշխատանքային օր), ճիշտ գործարքի նկարագրությամբ։ Կրկնակի գանձում չկա։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Վերջնական ֆինանսական արդյունքի ճշգրտություն</t>
+    <t xml:space="preserve">BRD TTZV-6011 §11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ցանկացած թեստային հաճախորդ՝ պարտատոմսով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բացել հաշվարկի մանրամասն հաշվետվությունը / log-ը։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հնարավոր է տեսնել, թե որ հաշիվներն են ներառվել (ներառյալ պարտատոմսի հաշիվը) և դրանց մասնաբաժինը միջին մնացորդում (հետագծելիություն, տես Q8)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Աուդիտի և վեճերի լուծման հնարավորություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-22</t>
   </si>
   <si>
-    <t xml:space="preserve">TTZV-4447 STATUS Քայլ 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդների խումբ՝ պարտատոմսով որակավորվող և չորակավորվող։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ստուգել ՍԾՎ/ՍԾԶՎ-ին տրամադրվող անհամապատասխան հաճախորդների ցուցակը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ցուցակում ներառված են միայն այն հաճախորդները, որոնք պարտատոմսը հաշվի առնելով էլ չեն համապատասխանում։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Արտահանման ճշգրտություն</t>
+    <t xml:space="preserve">E. Ռեգրեսիա</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 (ամբողջ տրամաբանություն)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդներ առանց պարտատոմսի, որոնք ծածկում են TTZV-4447-ի բոլոր ճյուղերը (Քայլ 1/2/3, աշխատավարձով և մնացորդով)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել ամսական հաշվարկը (1-ին աշխատանքային օրվա ռեժիմով) թեստային հաճախորդի համար։ Բացել հաշվարկի արդյունքը / log-ը և գանձման գործարքը LSoft-ում։ Համեմատել փոփոխությունից առաջ ստացված արդյունքի հետ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Արդյունքները (վճար, ցուցակ, ծանուցում) նույնն են, ինչ փոփոխությունից առաջ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոփոխությունը չի խախտել գործող լուծումը</t>
   </si>
   <si>
     <t xml:space="preserve">TC-23</t>
   </si>
   <si>
-    <t xml:space="preserve">TTZV-4447 Scope (ծանուցում)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդներ, որոնք որակավորվում են միայն պարտատոմսի շնորհիվ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ստուգել ծանուցումների ուղարկման log-ը և ՍԾԶՎ-ին տրամադրվող ցուցակը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Այդ հաճախորդները ծանուցում ՉԵՆ ստանում և ցուցակում ներառված չեն։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդի հաղորդակցության ճշգրտություն</t>
+    <t xml:space="preserve">Աշխատավարձին հավասարեցված եկամուտներ (թոշակ, նպաստ, շահաբաժին և այլն) + պարտատոմս։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Աշխատավարձի չափանիշի ստուգումը չի փոխվել։ Պարտատոմսի մարումը / արժեկտրոնը ՉԻ դիտարկվում որպես աշխատավարձ, եթե այլ բան համաձայնեցված չէ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Եկամտի և մնացորդի չափանիշների տարանջատում</t>
   </si>
   <si>
     <t xml:space="preserve">TC-24</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011 §11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ցանկացած թեստային հաճախորդ՝ պարտատոմսով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բացել հաշվարկի մանրամասն հաշվետվությունը / log-ը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հնարավոր է տեսնել, թե որ հաշիվներն են ներառվել (ներառյալ պարտատոմսի հաշիվը) և դրանց մասնաբաժինը միջին մնացորդում (հետագծելիություն, տես Q8)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Աուդիտի և վեճերի լուծման հնարավորություն</t>
+    <t xml:space="preserve">Այլ փաթեթներ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 §4 (Optimal, Advanced)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimal / Advanced փաթեթով և առանց փաթեթի հաճախորդներ՝ պարտատոմսով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել համապատասխան գանձման գործընթացները։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Այլ փաթեթների հաշվարկը չի փոխվել (փոփոխությունը վերաբերում է միայն PLUS CLUB, PLUS DIGITAL, STATUS փաթեթներին)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Շրջանակից դուրս ազդեցության բացակայություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-25</t>
   </si>
   <si>
-    <t xml:space="preserve">E. Ռեգրեսիա</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 (ամբողջ տրամաբանություն)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդներ առանց պարտատոմսի, որոնք ծածկում են TTZV-4447-ի բոլոր ճյուղերը (Քայլ 1/2/3, աշխատավարձով և մնացորդով)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել ամսական հաշվարկը (1-ին աշխատանքային օրվա ռեժիմով) թեստային հաճախորդի համար։ Բացել հաշվարկի արդյունքը / log-ը և գանձման գործարքը LSoft-ում։ Համեմատել փոփոխությունից առաջ ստացված արդյունքի հետ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Արդյունքները (վճար, ցուցակ, ծանուցում) նույնն են, ինչ փոփոխությունից առաջ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոփոխությունը չի խախտել գործող լուծումը</t>
+    <t xml:space="preserve">TTZV-4447 (սակագների ճկունություն)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոխել մեկ փաթեթի սակագինը թեստային միջավայրում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոփոխությունը կիրառվում է միայն տվյալ փաթեթի վրա, պարտատոմսի ներառումը շարունակում է աշխատել։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Սակագների ճկունությունը պահպանված է</t>
   </si>
   <si>
     <t xml:space="preserve">TC-26</t>
   </si>
   <si>
-    <t xml:space="preserve">Աշխատավարձին հավասարեցված եկամուտներ (թոշակ, նպաստ, շահաբաժին և այլն) + պարտատոմս։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Աշխատավարձի չափանիշի ստուգումը չի փոխվել։ Պարտատոմսի մարումը / արժեկտրոնը ՉԻ դիտարկվում որպես աշխատավարձ, եթե այլ բան համաձայնեցված չէ (տես Q2)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Եկամտի և մնացորդի չափանիշների տարանջատում</t>
+    <t xml:space="preserve">TTZV-4447 Քայլ 1 (ժամանակացույց)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ամբողջական պաշարային (batch) գործարկում իրականին մոտ ծավալով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել ամսական հաշվարկը բոլոր փաթեթային հաճախորդների համար։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկվում է ամսվա 1-ին աշխատանքային օրը, ավարտվում է առանց սխալների, տևողությունը էականորեն չի աճել նախորդ տարբերակի համեմատ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Կատարողականություն և կայունություն</t>
   </si>
   <si>
     <t xml:space="preserve">TC-27</t>
   </si>
   <si>
-    <t xml:space="preserve">Այլ փաթեթներ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 §4 (Optimal, Advanced)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optimal / Advanced փաթեթով և առանց փաթեթի հաճախորդներ՝ պարտատոմսով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել համապատասխան գանձման գործընթացները։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Այլ փաթեթների հաշվարկը չի փոխվել (փոփոխությունը վերաբերում է միայն PLUS CLUB, PLUS DIGITAL, STATUS փաթեթներին)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Շրջանակից դուրս ազդեցության բացակայություն</t>
+    <t xml:space="preserve">F. Բիզնես հաստատում</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Իրական (կամ անանունացված) պարտատոմս ունեցող 10–20 հաճախորդների նմուշ, յուրաքանչյուր փաթեթից։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ՍԾԶՎ/ՑՎՎ-ն ձեռքով հաշվարկում է միջին մնացորդը և սպասվող վճարը, համեմատում համակարգի արդյունքի հետ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բոլոր նմուշային հաճախորդների համար համակարգի և ձեռքով հաշվարկի արդյունքները համընկնում են։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բիզնեսի կողմից լուծման հաստատում</t>
   </si>
   <si>
     <t xml:space="preserve">TC-28</t>
   </si>
   <si>
-    <t xml:space="preserve">TTZV-4447 (սակագների ճկունություն)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոխել մեկ փաթեթի սակագինը թեստային միջավայրում։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոփոխությունը կիրառվում է միայն տվյալ փաթեթի վրա, պարտատոմսի ներառումը շարունակում է աշխատել։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Սակագների ճկունությունը պահպանված է</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 Քայլ 1 (ժամանակացույց)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ամբողջական պաշարային (batch) գործարկում իրականին մոտ ծավալով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել ամսական հաշվարկը բոլոր փաթեթային հաճախորդների համար։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկվում է ամսվա 1-ին աշխատանքային օրը, ավարտվում է առանց սխալների, տևողությունը էականորեն չի աճել նախորդ տարբերակի համեմատ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Կատարողականություն և կայունություն</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F. Բիզնես հաստատում</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Իրական (կամ անանունացված) պարտատոմս ունեցող 10–20 հաճախորդների նմուշ, յուրաքանչյուր փաթեթից։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ՍԾԶՎ/ՑՎՎ-ն ձեռքով հաշվարկում է միջին մնացորդը և սպասվող վճարը, համեմատում համակարգի արդյունքի հետ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բոլոր նմուշային հաճախորդների համար համակարգի և ձեռքով հաշվարկի արդյունքները համընկնում են։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բիզնեսի կողմից լուծման հաստատում</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-31</t>
-  </si>
-  <si>
     <t xml:space="preserve">Բոլոր նախորդ դեպքերը Passed են, բաց հարցերը փակված են։</t>
   </si>
   <si>
@@ -747,58 +711,70 @@
     <t xml:space="preserve">Պատասխան / որոշում</t>
   </si>
   <si>
-    <t xml:space="preserve">Ով է պատասխանել, ամսաթիվ</t>
+    <t xml:space="preserve">Ամսաթիվ</t>
   </si>
   <si>
     <t xml:space="preserve">Q1</t>
   </si>
   <si>
-    <t xml:space="preserve">Ինչպե՞ս է հաշվարկվում պարտատոմսի հաշվի «միջին մնացորդը»՝ օրական միջին, ամսվա վերջի մնացորդների միջին, թե այլ կերպ։ Նույն մեթոդաբանությունն է, ինչ ավանդներինը՞։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Առանց դրա հնարավոր չէ սահմանել ակնկալվող թիվը միջնամասում բացված/մարված պարտատոմսերի համար։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-14, TC-15</t>
+    <t xml:space="preserve">Ինչպե՞ս է հաշվարկվում պարտատոմսի հաշվի միջին մնացորդը, եթե պարտատոմսը ձեռք է բերվել կամ մարվել 3 ամսյա ժամանակահատվածի ընթացքում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ակնկալվող թիվը միջնամասում բացված / մարված պարտատոմսերի համար։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— (դեպքերը հանված են)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Չդիտարկել – թեստավորման շրջանակից դուրս է</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փակված</t>
   </si>
   <si>
     <t xml:space="preserve">Q2</t>
   </si>
   <si>
-    <t xml:space="preserve">Պարտատոմսը ո՞ր արժեքով է հաշվառվում՝ անվանական, ձեռքբերման, շուկայական արժեքով, թե ներառված է կուտակված արժեկտրոնը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Որոշում է ակնկալվող մնացորդը բոլոր պարտատոմսային դեպքերում։ Նաև՝ արժեկտրոնի վճարումը համարվու՞մ է աշխատավարձին հավասարեցված եկամուտ (շահաբաժինները համարվում են)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-01–TC-13, TC-26</t>
+    <t xml:space="preserve">Պարտատոմսը ո՞ր արժեքով է հաշվառվում՝ անվանական, ձեռքբերման, շուկայական, թե կուտակված արժեկտրոնով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Որոշում է ակնկալվող մնացորդը բոլոր պարտատոմսային դեպքերում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-01–TC-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Անվանական արժեքով։ Կուտակված արժեկտրոնը և ձեռքբերման / շուկայական արժեքը չեն դիտարկվում։</t>
   </si>
   <si>
     <t xml:space="preserve">Q3</t>
   </si>
   <si>
-    <t xml:space="preserve">Արտարժութային պարտատոմսերը ո՞ր փոխարժեքով (ԿԲ, բանկի) և ո՞ր ամսաթվով են փոխարկվում ՀՀԴ-ի։</t>
+    <t xml:space="preserve">Արտարժութային պարտատոմսերը ո՞ր փոխարժեքով և ո՞ր ամսաթվով են փոխարկվում ՀՀԴ-ի։</t>
   </si>
   <si>
     <t xml:space="preserve">Ակնկալվող ՀՀԴ գումարի հաշվարկ։</t>
   </si>
   <si>
+    <t xml:space="preserve">— (դեպքը հանված է)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q4</t>
   </si>
   <si>
-    <t xml:space="preserve">Ո՞ր հաշվի տեսակներն / հաշվեկշռային հաշիվներն են LSoft-ում համարվում «պարտատոմսի հաշիվ» (պահառության հաշիվ, դրամական հաշիվ պարտատոմսերի համար)։ Միայն Արդշինբանկի թողարկած, թե՞ նաև երրորդ կողմի պարտատոմսեր։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Սահմանում է շրջանակը և TC-20-ի ակնկալվող արդյունքը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-19, TC-20</t>
+    <t xml:space="preserve">Ո՞ր հաշվի տեսակներն են LSoft-ում համարվում «պարտատոմսի հաշիվ»։ Միայն Արդշինբանկի, թե՞ նաև երրորդ կողմի պարտատոմսեր։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Շրջանակի սահմանում։</t>
   </si>
   <si>
     <t xml:space="preserve">Q5</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS Քայլ 2-ում և PLUS Քայլ 2-ում «մնացորդը» նույն 3 ամսյա միջին մնացորդն է՞, թե ընթացիկ մնացորդը։</t>
+    <t xml:space="preserve">STATUS և PLUS փաթեթների Քայլ 2-ում «մնացորդը» նույն 3 ամսյա միջին մնացորդն է՞, թե ընթացիկ մնացորդը։</t>
   </si>
   <si>
     <t xml:space="preserve">Հիմնական BRD-ում (TTZV-4447) ձևակերպումը միանշանակ չէ։ Թեստային դեպքերը ենթադրում են 3 ամսյա միջին։</t>
@@ -807,22 +783,25 @@
     <t xml:space="preserve">TC-04, TC-06, TC-08, TC-09, TC-12, TC-13</t>
   </si>
   <si>
+    <t xml:space="preserve">Բաց</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q6</t>
   </si>
   <si>
-    <t xml:space="preserve">Ո՞ր ամսվա հաշվարկից է կիրառվում փոփոխությունը, և պե՞տք է արդյոք վերահաշվարկ / փոխհատուցում նախորդ ամիսների համար։</t>
+    <t xml:space="preserve">Ո՞ր ամսվա հաշվարկից է կիրառվում փոփոխությունը, և պե՞տք է արդյոք վերահաշվարկ նախորդ ամիսների համար։</t>
   </si>
   <si>
     <t xml:space="preserve">Ազդում է արտադրական ստուգման և հաճախորդների բողոքների վրա։</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-25, TC-30</t>
+    <t xml:space="preserve">TC-22, TC-27</t>
   </si>
   <si>
     <t xml:space="preserve">Q7</t>
   </si>
   <si>
-    <t xml:space="preserve">Jira հղումների ճշտում․ PDF արտահանման ժամանակ տողատակի համարները կցվել են հայտի համարներին (TTZV-60111 → TTZV-6011, TTZV-44472/44474 → TTZV-4447, LSBANK-9943/9945 → LSBANK-994)։ Հաստատել ճիշտ համարները։</t>
+    <t xml:space="preserve">Jira հղումների ճշտում․ PDF արտահանման ժամանակ տողատակի համարները կցվել էին հայտի համարներին (TTZV-60111, TTZV-44472/44474, LSBANK-9943/9945)։</t>
   </si>
   <si>
     <t xml:space="preserve">Հետագծելիություն BRD ↔ թեստ ↔ Jira։</t>
@@ -831,43 +810,46 @@
     <t xml:space="preserve">Ամփոփում</t>
   </si>
   <si>
+    <t xml:space="preserve">Այո, հաստատված է․ ճիշտ համարներն են TTZV-6011, TTZV-4447, LSBANK-994։</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q8</t>
   </si>
   <si>
     <t xml:space="preserve">Պե՞տք է արդյոք հաշվետվությունում / log-ում առանձին ցույց տալ պարտատոմսի մասնաբաժինը։ BRD-ում պահանջ չկա։</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-24-ը կարող է լինել «nice to have»։</t>
+    <t xml:space="preserve">TC-21-ը կարող է լինել «nice to have»։</t>
   </si>
   <si>
     <t xml:space="preserve">Q9</t>
   </si>
   <si>
-    <t xml:space="preserve">Երկու BRD-ում էլ RACI մատրիցը լրացված չէ։ Ո՞վ է վերջնական հաստատողը (Accountable)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Պետք է նշել «Ամփոփում» թերթի Sign-off բաժնում։</t>
+    <t xml:space="preserve">Երկու BRD-ում էլ RACI մատրիցը լրացված չէ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Վերջնական հաստատողի սահմանում։</t>
   </si>
   <si>
     <t xml:space="preserve">Q10</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD TTZV-6011-ի ամսաթիվը (27 Sep 2023) ավելի վաղ է, քան հիմնական BRD-ինը (07 Aug 2025)։ Ճշտել ամսաթիվը և փաստաթղթի կարգավիճակը (Document Status դաշտում գրված է «STATUS»)։</t>
+    <t xml:space="preserve">BRD TTZV-6011-ի ամսաթիվը (27 Sep 2023) ավելի վաղ է, քան հիմնական BRD-ինը (07 Aug 2025), Document Status դաշտում գրված է «STATUS»։</t>
   </si>
   <si>
     <t xml:space="preserve">Փաստաթղթի վավերականություն։</t>
   </si>
   <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q11</t>
   </si>
   <si>
-    <t xml:space="preserve">BRD §6–8, §10 (Սահմանափակումներ, Կախվածություններ, Ռիսկեր, Համակարգեր) դատարկ են։ Հաստատել՝ LSoft, ինչպես հիմնական BRD-ում։</t>
+    <t xml:space="preserve">BRD §6–8, §10 (Սահմանափակումներ, Կախվածություններ, Ռիսկեր, Համակարգեր) դատարկ են։</t>
   </si>
   <si>
     <t xml:space="preserve">Ինտեգրացիոն թեստերի շրջանակ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
   </si>
 </sst>
 </file>
@@ -943,7 +925,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -960,6 +942,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1012,7 +1006,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1070,6 +1064,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1390,7 +1392,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1451,178 +1453,178 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>17</v>
-      </c>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="7" t="n">
-        <f aca="false">COUNTA('Թեստային դեպքեր'!A2:A200)</f>
-        <v>31</v>
+      <c r="A15" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B16" s="7" t="n">
+        <f aca="false">COUNTA('Թեստային դեպքեր'!A2:A200)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Passed")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="7" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Failed")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="7" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="7" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Not run")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="7" t="n">
-        <f aca="false">B15-SUM(B16:B19)</f>
-        <v>31</v>
-      </c>
-    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="8" t="n">
-        <f aca="false">COUNTIFS('Թեստային դեպքեր'!D2:D200,"Կրիտիկական",'Թեստային դեպքեր'!J2:J200,"&lt;&gt;Passed")</f>
-        <v>12</v>
+      <c r="A21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <f aca="false">B16-SUM(B17:B20)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="2" t="str">
-        <f aca="false">IF(B15=0,"",IF(AND(B16=B15),"Ընդունված է – բոլոր դեպքերը Passed","Չի ընդունված – առկա են չանցած/չկատարված դեպքեր"))</f>
+        <v>26</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <f aca="false">COUNTIFS('Թեստային դեպքեր'!D2:D200,"Կրիտիկական",'Թեստային դեպքեր'!J2:J200,"&lt;&gt;Passed")</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <f aca="false">IF(B16=0,"",IF(AND(B17=B16),"Ընդունված է – բոլոր դեպքերը Passed","Չի ընդունված – առկա են չանցած/չկատարված դեպքեր"))</f>
         <v>Չի ընդունված – առկա են չանցած/չկատարված դեպքեր</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="9" t="s">
+      <c r="A25" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="10"/>
+      <c r="B26" s="9" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B31" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B32" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
         <v>40</v>
       </c>
@@ -1630,7 +1632,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>42</v>
       </c>
@@ -1638,7 +1640,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
         <v>44</v>
       </c>
@@ -1646,12 +1648,20 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1673,7 +1683,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1694,78 +1704,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J2" s="14"/>
       <c r="K2" s="14"/>
@@ -1776,31 +1786,31 @@
     </row>
     <row r="3" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
@@ -1811,31 +1821,31 @@
     </row>
     <row r="4" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
@@ -1846,31 +1856,31 @@
     </row>
     <row r="5" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
@@ -1881,31 +1891,31 @@
     </row>
     <row r="6" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
@@ -1916,31 +1926,31 @@
     </row>
     <row r="7" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C7" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="I7" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>87</v>
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
@@ -1951,31 +1961,31 @@
     </row>
     <row r="8" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -1986,31 +1996,31 @@
     </row>
     <row r="9" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
@@ -2021,31 +2031,31 @@
     </row>
     <row r="10" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
@@ -2056,31 +2066,31 @@
     </row>
     <row r="11" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
@@ -2091,31 +2101,31 @@
     </row>
     <row r="12" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
@@ -2126,31 +2136,31 @@
     </row>
     <row r="13" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
@@ -2161,31 +2171,31 @@
     </row>
     <row r="14" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
@@ -2194,33 +2204,33 @@
       <c r="N14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J15" s="14"/>
       <c r="K15" s="14"/>
@@ -2231,31 +2241,31 @@
     </row>
     <row r="16" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
@@ -2266,31 +2276,31 @@
     </row>
     <row r="17" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>148</v>
+        <v>75</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
@@ -2301,31 +2311,31 @@
     </row>
     <row r="18" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
@@ -2336,31 +2346,31 @@
     </row>
     <row r="19" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>153</v>
+        <v>67</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>73</v>
+        <v>161</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>75</v>
+        <v>163</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
@@ -2369,33 +2379,33 @@
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>75</v>
+        <v>169</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
@@ -2404,33 +2414,33 @@
       <c r="N20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>75</v>
+        <v>175</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
@@ -2439,33 +2449,33 @@
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>65</v>
+        <v>145</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
@@ -2474,33 +2484,33 @@
       <c r="N22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
@@ -2509,33 +2519,33 @@
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>185</v>
+        <v>118</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>187</v>
+        <v>77</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
@@ -2544,33 +2554,33 @@
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>64</v>
+        <v>196</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
@@ -2579,33 +2589,33 @@
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>65</v>
+        <v>145</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>200</v>
+        <v>77</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
@@ -2614,33 +2624,33 @@
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>109</v>
+        <v>66</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>116</v>
+        <v>208</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>75</v>
+        <v>210</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="I27" s="13" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
@@ -2649,33 +2659,33 @@
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>208</v>
+        <v>66</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>209</v>
+        <v>179</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
@@ -2684,33 +2694,33 @@
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>197</v>
-      </c>
       <c r="C29" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>153</v>
+        <v>67</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>75</v>
+        <v>221</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
@@ -2719,113 +2729,8 @@
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="14"/>
-      <c r="O30" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="F31" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="I31" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
-      <c r="O31" s="14"/>
-    </row>
-    <row r="32" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="G32" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="H32" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="14"/>
-      <c r="O32" s="14"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O32"/>
+  <autoFilter ref="A1:O29"/>
   <conditionalFormatting sqref="J2:J200">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Passed"</formula>
@@ -2862,212 +2767,281 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="C3" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="E3" s="13" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-    </row>
-    <row r="3" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
+      <c r="F3" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-    </row>
-    <row r="5" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>244</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
+        <v>244</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
+      <c r="G6" s="16" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
-    </row>
-    <row r="8" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G7" s="16" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
+        <v>260</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
+      <c r="G9" s="16" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="E11" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
         <v>272</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="B12" s="13" t="s">
         <v>273</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-    </row>
-    <row r="11" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="C12" s="13" t="s">
         <v>274</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>275</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>276</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>278</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>279</v>
-      </c>
       <c r="D12" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
+        <v>271</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>235</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Close remaining open questions in TTZV-6011 test checklist
Step 1/2 balance is the quarterly average; effective-date question and
calculation-log case dropped as out of scope.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149r7b5293oK3v6EmbinnuA
</commit_message>
<xml_diff>
--- a/TTZV-6011_Test_Checklist.xlsx
+++ b/TTZV-6011_Test_Checklist.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Բաց հարցեր" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Թեստային դեպքեր'!$A$1:$O$29</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Թեստային դեպքեր'!$A$1:$O$28</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="272">
   <si>
     <t xml:space="preserve">Թեստավորման ստուգաթերթ – PLUS CLUB, PLUS DIGITAL, STATUS փաթեթների միջին մնացորդի հաշվարկի մեջ պարտատոմսի հաշվի մնացորդի ներառում</t>
   </si>
@@ -72,6 +72,12 @@
     <t xml:space="preserve">Անվանական արժեք (համաձայնեցված 16.10.2026, տես «Բաց հարցեր» Q2)</t>
   </si>
   <si>
+    <t xml:space="preserve">Մնացորդի ցուցանիշը Քայլ 1 և Քայլ 2-ում</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Եռամսյակային միջին մնացորդ (համաձայնեցված 16.10.2026, տես «Բաց հարցեր» Q5)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Թեստային միջավայր</t>
   </si>
   <si>
@@ -174,7 +180,7 @@
     <t xml:space="preserve">Թեստային տվյալներ</t>
   </si>
   <si>
-    <t xml:space="preserve">Բոլոր գումարները ՀՀԴ են։ «Միջին մնացորդ»-ը վերջին 3 ամսվա միջինն է։ Պարտատոմսի գումարները նշված են անվանական արժեքով։ Պարզության համար թեստային տվյալներում մնացորդները պահել հաստատուն ամբողջ ժամանակահատվածում, եթե դեպքը այլ բան չի պահանջում։</t>
+    <t xml:space="preserve">Բոլոր գումարները ՀՀԴ են։ «Միջին մնացորդ»-ը վերջին 3 ամսվա (եռամսյակային) միջինն է և կիրառվում է ինչպես Քայլ 1-ի, այնպես էլ Քայլ 2-ի ստուգման համար։ Պարտատոմսի գումարները նշված են անվանական արժեքով։ Պարզության համար թեստային տվյալներում մնացորդները պահել հաստատուն ամբողջ ժամանակահատվածում, եթե դեպքը այլ բան չի պահանջում։</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -564,129 +570,114 @@
     <t xml:space="preserve">TC-21</t>
   </si>
   <si>
+    <t xml:space="preserve">E. Ռեգրեսիա</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 (ամբողջ տրամաբանություն)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Հաճախորդներ առանց պարտատոմսի, որոնք ծածկում են TTZV-4447-ի բոլոր ճյուղերը (Քայլ 1/2/3, աշխատավարձով և մնացորդով)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել ամսական հաշվարկը (1-ին աշխատանքային օրվա ռեժիմով) թեստային հաճախորդի համար։ Բացել հաշվարկի արդյունքը / log-ը և գանձման գործարքը LSoft-ում։ Համեմատել փոփոխությունից առաջ ստացված արդյունքի հետ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Արդյունքները (վճար, ցուցակ, ծանուցում) նույնն են, ինչ փոփոխությունից առաջ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոփոխությունը չի խախտել գործող լուծումը</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Աշխատավարձին հավասարեցված եկամուտներ (թոշակ, նպաստ, շահաբաժին և այլն) + պարտատոմս։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Աշխատավարձի չափանիշի ստուգումը չի փոխվել։ Պարտատոմսի մարումը / արժեկտրոնը ՉԻ դիտարկվում որպես աշխատավարձ, եթե այլ բան համաձայնեցված չէ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Եկամտի և մնացորդի չափանիշների տարանջատում</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Այլ փաթեթներ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 §4 (Optimal, Advanced)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimal / Advanced փաթեթով և առանց փաթեթի հաճախորդներ՝ պարտատոմսով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել համապատասխան գանձման գործընթացները։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Այլ փաթեթների հաշվարկը չի փոխվել (փոփոխությունը վերաբերում է միայն PLUS CLUB, PLUS DIGITAL, STATUS փաթեթներին)։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Շրջանակից դուրս ազդեցության բացակայություն</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 (սակագների ճկունություն)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոխել մեկ փաթեթի սակագինը թեստային միջավայրում։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Փոփոխությունը կիրառվում է միայն տվյալ փաթեթի վրա, պարտատոմսի ներառումը շարունակում է աշխատել։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Սակագների ճկունությունը պահպանված է</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TTZV-4447 Քայլ 1 (ժամանակացույց)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ամբողջական պաշարային (batch) գործարկում իրականին մոտ ծավալով։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկել ամսական հաշվարկը բոլոր փաթեթային հաճախորդների համար։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Գործարկվում է ամսվա 1-ին աշխատանքային օրը, ավարտվում է առանց սխալների, տևողությունը էականորեն չի աճել նախորդ տարբերակի համեմատ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Կատարողականություն և կայունություն</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F. Բիզնես հաստատում</t>
+  </si>
+  <si>
     <t xml:space="preserve">BRD TTZV-6011 §11</t>
   </si>
   <si>
-    <t xml:space="preserve">Ցանկացած թեստային հաճախորդ՝ պարտատոմսով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բացել հաշվարկի մանրամասն հաշվետվությունը / log-ը։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հնարավոր է տեսնել, թե որ հաշիվներն են ներառվել (ներառյալ պարտատոմսի հաշիվը) և դրանց մասնաբաժինը միջին մնացորդում (հետագծելիություն, տես Q8)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Աուդիտի և վեճերի լուծման հնարավորություն</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E. Ռեգրեսիա</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 (ամբողջ տրամաբանություն)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Հաճախորդներ առանց պարտատոմսի, որոնք ծածկում են TTZV-4447-ի բոլոր ճյուղերը (Քայլ 1/2/3, աշխատավարձով և մնացորդով)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել ամսական հաշվարկը (1-ին աշխատանքային օրվա ռեժիմով) թեստային հաճախորդի համար։ Բացել հաշվարկի արդյունքը / log-ը և գանձման գործարքը LSoft-ում։ Համեմատել փոփոխությունից առաջ ստացված արդյունքի հետ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Արդյունքները (վճար, ցուցակ, ծանուցում) նույնն են, ինչ փոփոխությունից առաջ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոփոխությունը չի խախտել գործող լուծումը</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Աշխատավարձին հավասարեցված եկամուտներ (թոշակ, նպաստ, շահաբաժին և այլն) + պարտատոմս։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Աշխատավարձի չափանիշի ստուգումը չի փոխվել։ Պարտատոմսի մարումը / արժեկտրոնը ՉԻ դիտարկվում որպես աշխատավարձ, եթե այլ բան համաձայնեցված չէ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Եկամտի և մնացորդի չափանիշների տարանջատում</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Այլ փաթեթներ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 §4 (Optimal, Advanced)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optimal / Advanced փաթեթով և առանց փաթեթի հաճախորդներ՝ պարտատոմսով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել համապատասխան գանձման գործընթացները։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Այլ փաթեթների հաշվարկը չի փոխվել (փոփոխությունը վերաբերում է միայն PLUS CLUB, PLUS DIGITAL, STATUS փաթեթներին)։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Շրջանակից դուրս ազդեցության բացակայություն</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 (սակագների ճկունություն)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոխել մեկ փաթեթի սակագինը թեստային միջավայրում։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Փոփոխությունը կիրառվում է միայն տվյալ փաթեթի վրա, պարտատոմսի ներառումը շարունակում է աշխատել։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Սակագների ճկունությունը պահպանված է</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TTZV-4447 Քայլ 1 (ժամանակացույց)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ամբողջական պաշարային (batch) գործարկում իրականին մոտ ծավալով։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկել ամսական հաշվարկը բոլոր փաթեթային հաճախորդների համար։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Գործարկվում է ամսվա 1-ին աշխատանքային օրը, ավարտվում է առանց սխալների, տևողությունը էականորեն չի աճել նախորդ տարբերակի համեմատ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Կատարողականություն և կայունություն</t>
+    <t xml:space="preserve">Իրական (կամ անանունացված) պարտատոմս ունեցող 10–20 հաճախորդների նմուշ, յուրաքանչյուր փաթեթից։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ՍԾԶՎ/ՑՎՎ-ն ձեռքով հաշվարկում է միջին մնացորդը և սպասվող վճարը, համեմատում համակարգի արդյունքի հետ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բոլոր նմուշային հաճախորդների համար համակարգի և ձեռքով հաշվարկի արդյունքները համընկնում են։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Բիզնեսի կողմից լուծման հաստատում</t>
   </si>
   <si>
     <t xml:space="preserve">TC-27</t>
   </si>
   <si>
-    <t xml:space="preserve">F. Բիզնես հաստատում</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Իրական (կամ անանունացված) պարտատոմս ունեցող 10–20 հաճախորդների նմուշ, յուրաքանչյուր փաթեթից։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ՍԾԶՎ/ՑՎՎ-ն ձեռքով հաշվարկում է միջին մնացորդը և սպասվող վճարը, համեմատում համակարգի արդյունքի հետ։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բոլոր նմուշային հաճախորդների համար համակարգի և ձեռքով հաշվարկի արդյունքները համընկնում են։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Բիզնեսի կողմից լուծման հաստատում</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-28</t>
-  </si>
-  <si>
     <t xml:space="preserve">Բոլոր նախորդ դեպքերը Passed են, բաց հարցերը փակված են։</t>
   </si>
   <si>
@@ -783,7 +774,7 @@
     <t xml:space="preserve">TC-04, TC-06, TC-08, TC-09, TC-12, TC-13</t>
   </si>
   <si>
-    <t xml:space="preserve">Բաց</t>
+    <t xml:space="preserve">Եռամսյակային միջին մնացորդ (Քայլ 1-ի և Քայլ 2-ի համար նույն ցուցանիշն է)։</t>
   </si>
   <si>
     <t xml:space="preserve">Q6</t>
@@ -795,7 +786,7 @@
     <t xml:space="preserve">Ազդում է արտադրական ստուգման և հաճախորդների բողոքների վրա։</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-22, TC-27</t>
+    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">Q7</t>
@@ -819,7 +810,10 @@
     <t xml:space="preserve">Պե՞տք է արդյոք հաշվետվությունում / log-ում առանձին ցույց տալ պարտատոմսի մասնաբաժինը։ BRD-ում պահանջ չկա։</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-21-ը կարող է լինել «nice to have»։</t>
+    <t xml:space="preserve">Հետագծելիության պահանջ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ոչ, պահանջ չկա։</t>
   </si>
   <si>
     <t xml:space="preserve">Q9</t>
@@ -838,9 +832,6 @@
   </si>
   <si>
     <t xml:space="preserve">Փաստաթղթի վավերականություն։</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">Q11</t>
@@ -925,7 +916,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -948,12 +939,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1006,7 +991,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1068,10 +1053,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1392,7 +1373,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1461,178 +1442,178 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B13" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>19</v>
-      </c>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="7" t="n">
-        <f aca="false">COUNTA('Թեստային դեպքեր'!A2:A200)</f>
-        <v>28</v>
+      <c r="A16" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" s="7" t="n">
+        <f aca="false">COUNTA('Թեստային դեպքեր'!A2:A200)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Passed")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="7" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Failed")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="7" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="7" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Թեստային դեպքեր'!J2:J200,"Not run")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="7" t="n">
-        <f aca="false">B16-SUM(B17:B20)</f>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <f aca="false">B17-SUM(B18:B21)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="8" t="n">
+      <c r="B23" s="8" t="n">
         <f aca="false">COUNTIFS('Թեստային դեպքեր'!D2:D200,"Կրիտիկական",'Թեստային դեպքեր'!J2:J200,"&lt;&gt;Passed")</f>
         <v>13</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="2" t="str">
-        <f aca="false">IF(B16=0,"",IF(AND(B17=B16),"Ընդունված է – բոլոր դեպքերը Passed","Չի ընդունված – առկա են չանցած/չկատարված դեպքեր"))</f>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <f aca="false">IF(B17=0,"",IF(AND(B18=B17),"Ընդունված է – բոլոր դեպքերը Passed","Չի ընդունված – առկա են չանցած/չկատարված դեպքեր"))</f>
         <v>Չի ընդունված – առկա են չանցած/չկատարված դեպքեր</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="9" t="s">
+      <c r="A26" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="10"/>
+      <c r="B27" s="9" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B33" s="10"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
         <v>40</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>42</v>
       </c>
@@ -1640,7 +1621,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
         <v>44</v>
       </c>
@@ -1648,7 +1629,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>46</v>
       </c>
@@ -1656,12 +1637,20 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1683,7 +1672,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1704,78 +1693,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J2" s="14"/>
       <c r="K2" s="14"/>
@@ -1786,31 +1775,31 @@
     </row>
     <row r="3" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
@@ -1821,31 +1810,31 @@
     </row>
     <row r="4" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
@@ -1856,31 +1845,31 @@
     </row>
     <row r="5" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
@@ -1891,31 +1880,31 @@
     </row>
     <row r="6" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
@@ -1926,31 +1915,31 @@
     </row>
     <row r="7" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C7" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="I7" s="13" t="s">
         <v>91</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>89</v>
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
@@ -1961,31 +1950,31 @@
     </row>
     <row r="8" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -1996,31 +1985,31 @@
     </row>
     <row r="9" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
@@ -2031,31 +2020,31 @@
     </row>
     <row r="10" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
@@ -2066,31 +2055,31 @@
     </row>
     <row r="11" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
@@ -2101,31 +2090,31 @@
     </row>
     <row r="12" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
@@ -2136,31 +2125,31 @@
     </row>
     <row r="13" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
@@ -2171,31 +2160,31 @@
     </row>
     <row r="14" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
@@ -2206,31 +2195,31 @@
     </row>
     <row r="15" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J15" s="14"/>
       <c r="K15" s="14"/>
@@ -2241,31 +2230,31 @@
     </row>
     <row r="16" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
@@ -2276,31 +2265,31 @@
     </row>
     <row r="17" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
@@ -2311,31 +2300,31 @@
     </row>
     <row r="18" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
@@ -2346,31 +2335,31 @@
     </row>
     <row r="19" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
@@ -2381,31 +2370,31 @@
     </row>
     <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
@@ -2416,31 +2405,31 @@
     </row>
     <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
@@ -2449,33 +2438,33 @@
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>145</v>
+        <v>69</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
@@ -2484,27 +2473,27 @@
       <c r="N22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>67</v>
+        <v>114</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>188</v>
+        <v>79</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>189</v>
@@ -2519,33 +2508,33 @@
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
         <v>191</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>111</v>
+        <v>192</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>118</v>
+        <v>193</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>77</v>
+        <v>195</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
@@ -2554,33 +2543,33 @@
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>196</v>
+        <v>68</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
@@ -2589,33 +2578,33 @@
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>77</v>
+        <v>206</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
@@ -2626,31 +2615,31 @@
     </row>
     <row r="27" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>145</v>
+        <v>69</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="I27" s="13" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
@@ -2659,33 +2648,33 @@
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
@@ -2694,43 +2683,8 @@
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="H29" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="I29" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
-      <c r="O29" s="14"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O29"/>
+  <autoFilter ref="A1:O28"/>
   <conditionalFormatting sqref="J2:J200">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Passed"</formula>
@@ -2781,266 +2735,278 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E1" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>228</v>
-      </c>
       <c r="G1" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="G2" s="15" t="s">
         <v>232</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="E3" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>240</v>
-      </c>
       <c r="F3" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>244</v>
-      </c>
       <c r="E4" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="E6" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="16" t="s">
-        <v>252</v>
+      <c r="F6" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="16" t="s">
-        <v>252</v>
+      <c r="E7" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>257</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="E8" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>259</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>261</v>
-      </c>
       <c r="F8" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>263</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>264</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="16" t="s">
-        <v>252</v>
+      <c r="F9" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>267</v>
-      </c>
       <c r="D10" s="13" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>270</v>
-      </c>
       <c r="D11" s="13" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>